<commit_message>
📊 Horarios actualizados Línea 141 - 2001
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:47:16</t>
+          <t>Última actualización: 02:45:28</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:47:16</t>
+          <t>02:45:28</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:59</t>
+          <t>03:02</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:47:16</t>
+          <t>02:45:28</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>02:57</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>01:47:16</t>
+          <t>02:45:28</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>04:01</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,66 +569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:47:16</t>
+          <t>Última actualización: 02:45:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Hora_Scrap</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Hora_Llegada</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Linea</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Minutos</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Parada</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>01:47:16</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>02:57</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>215_ALUAR</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>70</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>LP1912</t>
+          <t>Total filas: 0</t>
         </is>
       </c>
     </row>
@@ -656,7 +604,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:47:16</t>
+          <t>Última actualización: 02:45:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2002
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:45:28</t>
+          <t>Última actualización: 03:39:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:45:28</t>
+          <t>03:39:32</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:45:28</t>
+          <t>03:39:32</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,23 +523,123 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:45:28</t>
+          <t>03:39:32</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:01</t>
+          <t>04:46</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>67</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03:39:32</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:53</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>74</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>03:39:32</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>05:11</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>03:39:32</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:22</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>103</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>03:39:32</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05:31</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>76</v>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D12" t="n">
+        <v>112</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -556,7 +656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,14 +669,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:45:28</t>
+          <t>Última actualización: 03:39:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>03:39:32</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>04:46</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>67</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -604,7 +756,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:45:28</t>
+          <t>Última actualización: 03:39:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2003
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,216 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:39:32</t>
+          <t>Última actualización: 04:31:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Hora_Scrap</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Hora_Llegada</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Linea</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Minutos</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Parada</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>03:39:32</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>03:48</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>14_ABASTO</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>9</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>LP1912</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>03:39:32</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>04:01</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>81_EL PELIGRO</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>22</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>LP1912</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>03:39:32</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>04:46</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>215_EL PELIGRO</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>67</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>LP1912</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>03:39:32</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>04:53</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>11_ETCHEVERRY</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>74</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>LP1912</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>03:39:32</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>05:11</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>17_ROMERO</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>92</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>LP1912</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>03:39:32</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>05:22</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>23_HERNANDEZ</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>103</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>LP1912</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>03:39:32</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>05:31</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>81_EL PELIGRO</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>112</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>LP1912</t>
+          <t>Total filas: 0</t>
         </is>
       </c>
     </row>
@@ -656,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -669,66 +467,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:39:32</t>
+          <t>Última actualización: 04:31:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Hora_Scrap</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Hora_Llegada</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Linea</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Minutos</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Parada</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>03:39:32</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>04:46</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>215_EL PELIGRO</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>67</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>LP1912</t>
+          <t>Total filas: 0</t>
         </is>
       </c>
     </row>
@@ -756,7 +502,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:39:32</t>
+          <t>Última actualización: 04:31:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2004
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:31:17</t>
+          <t>Última actualización: 05:03:28</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:31:17</t>
+          <t>Última actualización: 05:03:28</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:31:17</t>
+          <t>Última actualización: 05:03:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2005
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,541 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:03:28</t>
+          <t>Última actualización: 05:53:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>05:53</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06:03</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06:10</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>17</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06:24</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>31</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06:27</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>34</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>37</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>46</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:54</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>61</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>67</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07:03</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>70</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07:06</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>73</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07:13</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>80</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>87</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07:33</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>102</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>103</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>07:40</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>107</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>07:43</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>110</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>116</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -454,7 +981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,14 +994,116 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:03:28</t>
+          <t>Última actualización: 05:53:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06:10</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>17</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:06</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>73</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05:53:50</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -502,7 +1131,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:03:28</t>
+          <t>Última actualización: 05:53:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2006
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:53:50</t>
+          <t>Última actualización: 06:26:03</t>
         </is>
       </c>
     </row>
@@ -473,17 +473,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:53</t>
+          <t>06:26</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>06:31</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06:03</t>
+          <t>06:31</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06:10</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:24</t>
+          <t>06:51</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:27</t>
+          <t>06:54</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>07:01</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:04</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:54</t>
+          <t>07:07</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>07:14</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:03</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:06</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:13</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:33</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:49</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:57</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>07:40</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,12 +923,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>07:43</t>
+          <t>08:14</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,12 +948,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>07:49</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:53:50</t>
+          <t>Última actualización: 06:26:03</t>
         </is>
       </c>
     </row>
@@ -1035,12 +1035,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:10</t>
+          <t>06:51</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1060,12 +1060,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07:06</t>
+          <t>07:07</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1074,7 +1074,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>73</v>
+        <v>41</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1085,12 +1085,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:53:50</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1099,7 +1099,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>87</v>
+        <v>55</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1118,7 +1118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1131,14 +1131,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:53:50</t>
+          <t>Última actualización: 06:26:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>08:23</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>117</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2007
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:26:03</t>
+          <t>Última actualización: 06:57:47</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:26:03</t>
+          <t>Última actualización: 06:57:47</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1131,14 +1131,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:26:03</t>
+          <t>Última actualización: 06:57:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -1172,23 +1172,73 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>06:57:47</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>07:29</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>32</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>06:57:47</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>08:09</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>72</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>08:23</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D8" t="n">
         <v>117</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2008
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:57:47</t>
+          <t>Última actualización: 07:27:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:27:07</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -778,16 +778,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:27:07</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>71</v>
+        <v>3</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:27:07</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>78</v>
+        <v>8</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:27:07</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:49</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>83</v>
+        <v>9</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:27:07</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07:57</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>91</v>
+        <v>10</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:27:07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:42</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>94</v>
+        <v>15</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,12 +923,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:27:07</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>08:14</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>108</v>
+        <v>17</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,23 +948,398 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>22</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>06:26:03</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>07:57</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>91</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>07:58</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>31</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>33</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>34</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>08:03</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>36</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>08:14</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>47</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
         <is>
           <t>08:19</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>113</v>
-      </c>
-      <c r="E25" t="inlineStr">
+      <c r="D32" t="n">
+        <v>52</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>63</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>67</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>81</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>08:51</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>84</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>93</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>108</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>110</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>112</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -981,7 +1356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -994,14 +1369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:57:47</t>
+          <t>Última actualización: 07:27:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1102,6 +1477,131 @@
         <v>55</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07:27</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>67</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>81</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>93</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>112</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1131,7 +1631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:57:47</t>
+          <t>Última actualización: 07:27:07</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1722,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:27:07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1236,7 +1736,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>117</v>
+        <v>56</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2009
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:27:07</t>
+          <t>Última actualización: 07:57:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 49</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,12 +998,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>07:58</t>
+          <t>07:57</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>31</v>
+        <v>91</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:58</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1053,16 +1053,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1078,16 +1078,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>08:14</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>47</v>
+        <v>6</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:14</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>67</v>
+        <v>24</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:29</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>81</v>
+        <v>32</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1228,16 +1228,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>93</v>
+        <v>37</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>108</v>
+        <v>44</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>110</v>
+        <v>47</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,23 +1323,373 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>51</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>08:51</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>54</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>08:59</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>62</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>07:27:07</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>93</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>66</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>09:09</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>72</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>75</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>77</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>108</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>07:27:07</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>110</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>09:19</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D40" t="n">
-        <v>112</v>
-      </c>
-      <c r="E40" t="inlineStr">
+      <c r="D50" t="n">
+        <v>82</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>97</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>107</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>114</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>119</v>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1356,7 +1706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1369,14 +1719,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:27:07</t>
+          <t>Última actualización: 07:57:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1860,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1524,7 +1874,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1535,7 +1885,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1549,7 +1899,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1560,12 +1910,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:59</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1574,7 +1924,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1590,18 +1940,43 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>93</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>09:19</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>112</v>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D14" t="n">
+        <v>82</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1618,7 +1993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1631,14 +2006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:27:07</t>
+          <t>Última actualización: 07:57:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1722,23 +2097,98 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>08:10</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>13</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>08:23</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>56</v>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D9" t="n">
+        <v>26</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:58</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>61</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:57:31</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>119</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2010
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:57:31</t>
+          <t>Última actualización: 08:24:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 49</t>
+          <t>Total filas: 58</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:33</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:48</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>08:59</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>62</v>
+        <v>27</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,12 +1398,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:59</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>09:03</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>09:09</t>
+          <t>09:01</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>09:12</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>75</v>
+        <v>39</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>09:09</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>108</v>
+        <v>72</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,12 +1548,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>110</v>
+        <v>75</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1578,16 +1578,16 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>97</v>
+        <v>51</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>107</v>
+        <v>53</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>114</v>
+        <v>55</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,23 +1673,248 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>09:29</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>65</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>70</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>07:57:31</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>107</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>81</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>09:49</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>85</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>87</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
         <is>
           <t>09:56</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D54" t="n">
-        <v>119</v>
-      </c>
-      <c r="E54" t="inlineStr">
+      <c r="D60" t="n">
+        <v>92</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>100</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>105</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>116</v>
+      </c>
+      <c r="E63" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1706,7 +1931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1719,14 +1944,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:57:31</t>
+          <t>Última actualización: 08:24:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1860,7 +2085,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1874,7 +2099,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1885,7 +2110,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1899,7 +2124,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1935,7 +2160,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:27:07</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1949,7 +2174,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>93</v>
+        <v>36</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1960,7 +2185,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1974,9 +2199,34 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>100</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1993,7 +2243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2006,14 +2256,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:57:31</t>
+          <t>Última actualización: 08:24:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -2147,25 +2397,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>08:58</t>
+          <t>08:25</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>61</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
@@ -2177,18 +2427,43 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>08:58</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>61</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>09:56</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>119</v>
-      </c>
-      <c r="E11" t="inlineStr">
+      <c r="D12" t="n">
+        <v>92</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2011
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:24:08</t>
+          <t>Última actualización: 08:48:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 58</t>
+          <t>Total filas: 68</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1362,7 +1362,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1462,7 +1462,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1503,16 +1503,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>09:09</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>72</v>
+        <v>16</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>09:12</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>75</v>
+        <v>43</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1578,16 +1578,16 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>09:09</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1653,16 +1653,16 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>09:29</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1703,16 +1703,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>107</v>
+        <v>31</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:21</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>81</v>
+        <v>33</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>09:49</t>
+          <t>09:29</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>85</v>
+        <v>41</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:33</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>87</v>
+        <v>45</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>92</v>
+        <v>46</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1878,16 +1878,16 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>10:09</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>105</v>
+        <v>81</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1903,18 +1903,268 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
+          <t>09:49</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>85</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>08:48:26</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>63</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>08:48:26</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>68</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>08:48:26</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>76</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>08:48:26</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>80</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>105</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>08:48:26</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
           <t>10:20</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D63" t="n">
+      <c r="D69" t="n">
+        <v>92</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>08:48:26</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>102</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>08:48:26</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>104</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>08:48:26</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>106</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>08:48:26</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
         <v>116</v>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1944,7 +2194,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:24:08</t>
+          <t>Última actualización: 08:48:26</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2360,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2124,7 +2374,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2135,7 +2385,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2149,7 +2399,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2185,7 +2435,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2199,7 +2449,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2210,7 +2460,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2224,7 +2474,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2243,7 +2493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2256,14 +2506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:24:08</t>
+          <t>Última actualización: 08:48:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -2447,25 +2697,100 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>08:48:26</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:01</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>13</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>08:24:08</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>09:56</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D13" t="n">
         <v>92</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:48:26</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>83</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:48:26</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:22</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>94</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2012
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:48:26</t>
+          <t>Última actualización: 09:01:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 68</t>
+          <t>Total filas: 72</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1462,7 +1462,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1533,11 +1533,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>43</v>
+        <v>3</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,12 +1573,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:09</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1587,7 +1587,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>72</v>
+        <v>43</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1603,16 +1603,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>09:12</t>
+          <t>09:09</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>26</v>
+        <v>75</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,12 +1648,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1662,7 +1662,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,12 +1698,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>09:29</t>
+          <t>09:21</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1803,16 +1803,16 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>09:33</t>
+          <t>09:29</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:33</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,12 +1873,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>09:49</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>85</v>
+        <v>44</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:49</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>63</v>
+        <v>85</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>10:08</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,12 +2023,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>10:09</t>
+          <t>10:08</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>10:09</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:20</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>10:32</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2128,16 +2128,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,23 +2148,123 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>92</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>09:01:14</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>93</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>09:01:14</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
           <t>10:44</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D73" t="n">
+      <c r="D75" t="n">
+        <v>103</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>09:01:14</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>110</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>09:01:14</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
         <v>116</v>
       </c>
-      <c r="E73" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2194,7 +2294,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:48:26</t>
+          <t>Última actualización: 09:01:14</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2535,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2449,7 +2549,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2460,7 +2560,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2474,7 +2574,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2493,7 +2593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2506,14 +2606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:48:26</t>
+          <t>Última actualización: 09:01:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2797,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2711,7 +2811,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2747,48 +2847,73 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>70</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>09:01:14</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>10:22</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>94</v>
-      </c>
-      <c r="E15" t="inlineStr">
+      <c r="D16" t="n">
+        <v>81</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2013
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:01:14</t>
+          <t>Última actualización: 10:16:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 72</t>
+          <t>Total filas: 90</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>09:01:14</t>
+          <t>10:16:15</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:21</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>89</v>
+        <v>5</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>09:01:14</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>10:32</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,12 +2148,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>09:01:14</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>10:33</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2162,7 +2162,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>09:01:14</t>
+          <t>10:16:15</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:33</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>93</v>
+        <v>17</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>09:01:14</t>
+          <t>10:16:15</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:33</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>103</v>
+        <v>17</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>09:01:14</t>
+          <t>10:16:15</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>10:51</t>
+          <t>10:34</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>110</v>
+        <v>18</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,23 +2248,473 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>10:41</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>25</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
           <t>09:01:14</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>103</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>29</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>10:49</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>33</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>35</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>35</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
         <is>
           <t>10:57</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>41</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D77" t="n">
-        <v>116</v>
-      </c>
-      <c r="E77" t="inlineStr">
+      <c r="D84" t="n">
+        <v>41</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>48</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>11:07</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>51</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>52</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>63</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>65</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>76</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>11:33</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>77</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>89</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>11:51</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>95</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>11:56</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>100</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>108</v>
+      </c>
+      <c r="E95" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2281,7 +2731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2294,14 +2744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:01:14</t>
+          <t>Última actualización: 10:16:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2577,6 +3027,81 @@
         <v>63</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>63</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:33</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>77</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>89</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2606,7 +3131,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:01:14</t>
+          <t>Última actualización: 10:16:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2014
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:16:15</t>
+          <t>Última actualización: 10:57:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 90</t>
+          <t>Total filas: 107</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>10:16:15</t>
+          <t>10:57:29</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>10:58</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>10:16:15</t>
+          <t>10:57:29</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>11:07</t>
+          <t>10:58</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>10:16:15</t>
+          <t>10:57:29</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:01</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>10:16:15</t>
+          <t>10:57:29</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>11:19</t>
+          <t>11:03</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2553,16 +2553,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>11:21</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2578,16 +2578,16 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>11:07</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>76</v>
+        <v>51</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>10:16:15</t>
+          <t>10:57:29</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>11:33</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>77</v>
+        <v>11</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>10:16:15</t>
+          <t>10:57:29</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>11:11</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>89</v>
+        <v>14</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>10:16:15</t>
+          <t>10:57:29</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>11:51</t>
+          <t>11:19</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>10:16:15</t>
+          <t>10:57:29</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>11:56</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>100</v>
+        <v>23</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2703,18 +2703,443 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>65</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>35</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>11:33</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>36</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>11:33</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>36</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>44</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>47</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>10:16:15</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>89</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>11:49</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>52</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>11:51</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>54</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>11:56</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>59</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
           <t>12:04</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D95" t="n">
-        <v>108</v>
-      </c>
-      <c r="E95" t="inlineStr">
+      <c r="D105" t="n">
+        <v>67</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>71</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>12:19</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>82</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>83</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>95</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>97</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>101</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>12:51</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>114</v>
+      </c>
+      <c r="E112" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2731,7 +3156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2744,14 +3169,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:16:15</t>
+          <t>Última actualización: 10:57:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -3035,7 +3460,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10:16:15</t>
+          <t>10:57:29</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3049,7 +3474,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3060,7 +3485,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10:16:15</t>
+          <t>10:57:29</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3074,7 +3499,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>77</v>
+        <v>36</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3085,23 +3510,73 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>47</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>10:16:15</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>11:45</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D19" t="n">
         <v>89</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>97</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3118,7 +3593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3131,14 +3606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:16:15</t>
+          <t>Última actualización: 10:57:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -3441,6 +3916,56 @@
       <c r="E16" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:56</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>59</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>119</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2015
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E112"/>
+  <dimension ref="A1:E123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:57:29</t>
+          <t>Última actualización: 11:27:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 107</t>
+          <t>Total filas: 118</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>11:27</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2753,16 +2753,16 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>11:33</t>
+          <t>11:32</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2803,16 +2803,16 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>11:41</t>
+          <t>11:33</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>10:16:15</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>89</v>
+        <v>14</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>11:49</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>10:16:15</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>11:51</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>11:56</t>
+          <t>11:49</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:51</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>67</v>
+        <v>24</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:56</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>12:19</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>82</v>
+        <v>34</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>12:20</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>83</v>
+        <v>36</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>95</v>
+        <v>37</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>97</v>
+        <v>41</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>101</v>
+        <v>52</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,23 +3123,298 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>53</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>65</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>67</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>67</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
           <t>10:57:29</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>101</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>12:47</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>80</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>10:57:29</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
         <is>
           <t>12:51</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
+      <c r="C118" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D112" t="n">
+      <c r="D118" t="n">
         <v>114</v>
       </c>
-      <c r="E112" t="inlineStr">
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>12:52</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>85</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>95</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>97</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>13:17</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>11X44_P_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>110</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>112</v>
+      </c>
+      <c r="E123" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3156,7 +3431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3169,14 +3444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:57:29</t>
+          <t>Última actualización: 11:27:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3485,12 +3760,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>11:33</t>
+          <t>11:27</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3499,7 +3774,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3515,16 +3790,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:33</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3535,12 +3810,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10:16:15</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3549,7 +3824,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>89</v>
+        <v>17</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3560,23 +3835,98 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>10:16:15</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>89</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>12:34</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="D21" t="n">
+        <v>67</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
         <v>97</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>112</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3593,7 +3943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3606,14 +3956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:57:29</t>
+          <t>Última actualización: 11:27:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -3922,7 +4272,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3936,7 +4286,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3947,7 +4297,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3961,11 +4311,61 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>104</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>115</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2016
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E123"/>
+  <dimension ref="A1:E134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:27:21</t>
+          <t>Última actualización: 11:56:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 118</t>
+          <t>Total filas: 129</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3062,7 +3062,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3112,7 +3112,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3137,7 +3137,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,12 +3198,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,12 +3223,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>101</v>
+        <v>67</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3253,16 +3253,16 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>12:47</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>10:57:29</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>12:51</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>114</v>
+        <v>40</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>10:57:29</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>12:52</t>
+          <t>12:38</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:47</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:51</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>97</v>
+        <v>55</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3378,16 +3378,16 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>12:52</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>110</v>
+        <v>85</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,23 +3398,298 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>61</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
           <t>11:27:21</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr">
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>95</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>67</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>97</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>77</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>13:17</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>11X44_P_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>81</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>13:18</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>82</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
         <is>
           <t>13:19</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr">
+      <c r="C130" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D123" t="n">
+      <c r="D130" t="n">
         <v>112</v>
       </c>
-      <c r="E123" t="inlineStr">
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>96</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>101</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>111</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>115</v>
+      </c>
+      <c r="E134" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3431,7 +3706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3444,14 +3719,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:27:21</t>
+          <t>Última actualización: 11:56:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -3860,12 +4135,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3874,7 +4149,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3890,7 +4165,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3899,7 +4174,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>97</v>
+        <v>67</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3910,23 +4185,123 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>67</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>11:27:21</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>97</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:18</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>82</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>13:19</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D26" t="n">
         <v>112</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>101</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3943,7 +4318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3956,14 +4331,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:27:21</t>
+          <t>Última actualización: 11:56:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4647,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -4286,7 +4661,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -4297,12 +4672,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -4311,7 +4686,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -4327,43 +4702,118 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>13:11</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>74</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>11:27:21</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>104</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>85</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>11:27:21</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>13:22</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="D23" t="n">
         <v>115</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2017
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E134"/>
+  <dimension ref="A1:E144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:56:47</t>
+          <t>Última actualización: 12:24:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 129</t>
+          <t>Total filas: 139</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3187,7 +3187,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>12:51</t>
+          <t>12:49</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,12 +3373,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>12:52</t>
+          <t>12:51</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -3387,7 +3387,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:52</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:52</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>95</v>
+        <v>28</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>13:03</t>
+          <t>12:53</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>11:56:46</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>97</v>
+        <v>61</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>77</v>
+        <v>38</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3528,16 +3528,16 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>13:19</t>
+          <t>13:07</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>112</v>
+        <v>43</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3603,16 +3603,16 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>13:37</t>
+          <t>13:17</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>101</v>
+        <v>53</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>111</v>
+        <v>54</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3678,18 +3678,268 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
+          <t>13:18</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>82</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>12:24:27</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>55</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>12:24:27</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>57</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>12:24:27</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>68</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>11:56:46</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>101</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>12:24:27</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>74</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>12:24:27</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>83</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>12:24:27</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
           <t>13:51</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr">
+      <c r="C141" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D134" t="n">
-        <v>115</v>
-      </c>
-      <c r="E134" t="inlineStr">
+      <c r="D141" t="n">
+        <v>87</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>12:24:27</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>95</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>12:24:27</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>112</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>12:24:27</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>113</v>
+      </c>
+      <c r="E144" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3706,7 +3956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3719,14 +3969,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:56:47</t>
+          <t>Última actualización: 12:24:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4410,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4174,7 +4424,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4210,7 +4460,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4224,7 +4474,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>97</v>
+        <v>40</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4260,7 +4510,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4274,7 +4524,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>112</v>
+        <v>55</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4302,6 +4552,31 @@
         <v>101</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>12:24:27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>74</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4318,7 +4593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4331,14 +4606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:56:47</t>
+          <t>Última actualización: 12:24:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -4697,7 +4972,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -4711,7 +4986,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>89</v>
+        <v>32</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -4747,7 +5022,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4761,7 +5036,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>104</v>
+        <v>47</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -4797,7 +5072,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4811,11 +5086,36 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>115</v>
+        <v>58</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>12:24:27</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>92</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2018
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E144"/>
+  <dimension ref="A1:E150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:24:27</t>
+          <t>Última actualización: 12:51:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 139</t>
+          <t>Total filas: 145</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>12:53</t>
+          <t>12:52</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:53</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3528,16 +3528,16 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>13:03</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>13:07</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>77</v>
+        <v>40</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>13:07</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,12 +3648,12 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>13:08</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3662,7 +3662,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3678,16 +3678,16 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>13:19</t>
+          <t>13:17</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>13:37</t>
+          <t>13:19</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>101</v>
+        <v>55</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>13:38</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>74</v>
+        <v>30</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>83</v>
+        <v>41</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>87</v>
+        <v>46</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3878,16 +3878,16 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:38</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>112</v>
+        <v>56</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,23 +3923,173 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>60</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>12:51:43</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>68</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>12:51:43</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>85</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>12:51:43</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
           <t>14:17</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr">
+      <c r="C147" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D144" t="n">
-        <v>113</v>
-      </c>
-      <c r="E144" t="inlineStr">
+      <c r="D147" t="n">
+        <v>86</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>12:51:43</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>87</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>12:51:43</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>14:32</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>101</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>12:51:43</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>14:38</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>107</v>
+      </c>
+      <c r="E150" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3956,7 +4106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3969,14 +4119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:24:27</t>
+          <t>Última actualización: 12:51:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -4435,7 +4585,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4449,7 +4599,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>67</v>
+        <v>12</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4485,7 +4635,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4499,7 +4649,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>82</v>
+        <v>27</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4535,7 +4685,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4549,7 +4699,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>101</v>
+        <v>46</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4577,6 +4727,31 @@
         <v>74</v>
       </c>
       <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>12:51:43</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>87</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4593,7 +4768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4606,14 +4781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:24:27</t>
+          <t>Última actualización: 12:51:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -4947,7 +5122,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -4961,7 +5136,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>59</v>
+        <v>4</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -4997,7 +5172,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -5011,7 +5186,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>74</v>
+        <v>19</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -5047,7 +5222,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:56:46</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5061,7 +5236,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>85</v>
+        <v>30</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -5114,6 +5289,31 @@
         <v>92</v>
       </c>
       <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>12:51:43</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>66</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2019
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E150"/>
+  <dimension ref="A1:E164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:51:43</t>
+          <t>Última actualización: 13:20:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 145</t>
+          <t>Total filas: 159</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:20</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3853,16 +3853,16 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>13:37</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>13:38</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3928,16 +3928,16 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:38</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>13:41</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>85</v>
+        <v>21</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>86</v>
+        <v>27</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>14:18</t>
+          <t>13:48</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>87</v>
+        <v>28</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>13:51</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>101</v>
+        <v>31</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,23 +4073,373 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>39</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>43</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
           <t>12:51:43</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr">
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>85</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>57</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>57</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>12:51:43</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>87</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>59</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>12:51:43</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>14:32</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>101</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>73</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
         <is>
           <t>14:38</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr">
+      <c r="C159" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D150" t="n">
-        <v>107</v>
-      </c>
-      <c r="E150" t="inlineStr">
+      <c r="D159" t="n">
+        <v>78</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>90</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>14:51</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>91</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>99</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>100</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>15:19</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>119</v>
+      </c>
+      <c r="E164" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4106,7 +4456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4119,14 +4469,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:51:43</t>
+          <t>Última actualización: 13:20:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -4685,21 +5035,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>13:37</t>
+          <t>13:20</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4710,12 +5060,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>13:38</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -4724,7 +5074,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -4735,23 +5085,123 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>18</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>12:51:43</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>14:18</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D30" t="n">
         <v>87</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>59</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>100</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:19</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>119</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4768,7 +5218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4781,14 +5231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:51:43</t>
+          <t>Última actualización: 13:20:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -5247,7 +5697,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5261,7 +5711,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -5316,6 +5766,81 @@
       <c r="E25" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>42</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>86</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>106</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2020
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E164"/>
+  <dimension ref="A1:E175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:20:14</t>
+          <t>Última actualización: 13:53:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 159</t>
+          <t>Total filas: 170</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3883,7 +3883,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4087,7 +4087,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,12 +4098,12 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -4112,7 +4112,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4153,16 +4153,16 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>14:18</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>14:19</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:18</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>101</v>
+        <v>25</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4278,16 +4278,16 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:19</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:21</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>78</v>
+        <v>28</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4353,16 +4353,16 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>99</v>
+        <v>45</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>100</v>
+        <v>54</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4428,18 +4428,293 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>90</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>13:53:51</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>14:51</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>58</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>13:53:51</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>14:52</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>59</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>13:53:51</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>66</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>13:53:51</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>66</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>100</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>13:53:51</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>85</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
           <t>15:19</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr">
+      <c r="C171" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D164" t="n">
+      <c r="D171" t="n">
         <v>119</v>
       </c>
-      <c r="E164" t="inlineStr">
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>13:53:51</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>105</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>13:53:51</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>108</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>13:53:51</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>114</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>13:53:51</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>15:51</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>118</v>
+      </c>
+      <c r="E175" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4456,7 +4731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4469,14 +4744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:20:14</t>
+          <t>Última actualización: 13:53:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5385,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5124,7 +5399,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>87</v>
+        <v>25</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5160,12 +5435,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -5174,7 +5449,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>100</v>
+        <v>66</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5190,18 +5465,68 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>100</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>13:53:51</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>85</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>15:19</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D35" t="n">
         <v>119</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5218,7 +5543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5231,14 +5556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:20:14</t>
+          <t>Última actualización: 13:53:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -5797,12 +6122,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>14:46</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -5811,7 +6136,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -5822,23 +6147,98 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>13:53:51</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>52</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>13:20:14</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>86</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>13:53:51</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>72</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>13:20:14</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>15:06</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D31" t="n">
         <v>106</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2021
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:53:51</t>
+          <t>Última actualización: 14:19:46</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4233,11 +4233,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4744,7 +4744,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:53:51</t>
+          <t>Última actualización: 14:19:46</t>
         </is>
       </c>
     </row>
@@ -5556,7 +5556,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:53:51</t>
+          <t>Última actualización: 14:19:46</t>
         </is>
       </c>
     </row>
@@ -6197,7 +6197,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>14:19:46</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6211,7 +6211,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2022
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E175"/>
+  <dimension ref="A1:E189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:19:46</t>
+          <t>Última actualización: 14:49:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 170</t>
+          <t>Total filas: 184</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4423,12 +4423,12 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>14:49:31</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>14:49</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>58</v>
+        <v>90</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>14:49:31</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>14:52</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>59</v>
+        <v>2</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4503,16 +4503,16 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:52</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>14:49:31</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>14:49:31</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>14:49:31</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>119</v>
+        <v>12</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>14:49:31</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>14:49:31</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>108</v>
+        <v>22</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4678,16 +4678,16 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>114</v>
+        <v>85</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,23 +4698,373 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>14:49:31</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
+          <t>15:19</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>30</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>34</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>15:33</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>44</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>46</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>49</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>52</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>58</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
           <t>15:51</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
+      <c r="C182" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D175" t="n">
+      <c r="D182" t="n">
+        <v>62</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>65</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>67</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>16:09</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>80</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>16:11</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>82</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>95</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>106</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>16:47</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
         <v>118</v>
       </c>
-      <c r="E175" t="inlineStr">
+      <c r="E189" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4731,7 +5081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4744,14 +5094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:19:46</t>
+          <t>Última actualización: 14:49:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -5435,7 +5785,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>14:49:31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5449,7 +5799,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5510,7 +5860,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>14:49:31</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -5524,9 +5874,34 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>119</v>
+        <v>30</v>
       </c>
       <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>95</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5543,7 +5918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5556,14 +5931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:19:46</t>
+          <t>Última actualización: 14:49:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -6241,6 +6616,31 @@
       <c r="E31" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>14:49:31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15:46</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>57</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2023
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E189"/>
+  <dimension ref="A1:E195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:49:31</t>
+          <t>Última actualización: 15:02:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 184</t>
+          <t>Total filas: 190</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4233,11 +4233,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>15:03</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>85</v>
+        <v>9</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,12 +4698,12 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4728,16 +4728,16 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:19</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>15:33</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:33</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4803,16 +4803,16 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:54</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>80</v>
+        <v>54</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:21</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,23 +5048,173 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
+          <t>15:02:46</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>81</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
           <t>14:49:31</t>
         </is>
       </c>
-      <c r="B189" t="inlineStr">
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>95</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>15:02:46</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>93</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>15:02:46</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
         <is>
           <t>16:47</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr">
+      <c r="C192" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D189" t="n">
-        <v>118</v>
-      </c>
-      <c r="E189" t="inlineStr">
+      <c r="D192" t="n">
+        <v>105</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>15:02:46</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>109</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>15:02:46</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>117</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>15:02:46</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>117</v>
+      </c>
+      <c r="E195" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5081,7 +5231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5094,14 +5244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:49:31</t>
+          <t>Última actualización: 15:02:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -5835,7 +5985,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5849,7 +5999,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -5885,23 +6035,73 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>15:02:46</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>81</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>14:49:31</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>16:24</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D36" t="n">
+      <c r="D37" t="n">
         <v>95</v>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>15:02:46</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>117</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5918,7 +6118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5931,14 +6131,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:49:31</t>
+          <t>Última actualización: 15:02:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -6572,7 +6772,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14:19:46</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6586,7 +6786,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -6622,23 +6822,98 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>15:02:46</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>43</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>14:49:31</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>15:46</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D32" t="n">
+      <c r="D33" t="n">
         <v>57</v>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>15:02:46</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>16:42</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>100</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>15:02:46</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>113</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2024
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:02:46</t>
+          <t>Última actualización: 15:56:34</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4233,11 +4233,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -5244,7 +5244,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:02:46</t>
+          <t>Última actualización: 15:56:34</t>
         </is>
       </c>
     </row>
@@ -6118,7 +6118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6131,14 +6131,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:02:46</t>
+          <t>Última actualización: 15:56:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -6897,23 +6897,48 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>15:02:46</t>
+          <t>15:56:34</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>16:43</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>47</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>15:56:34</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>16:55</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>113</v>
-      </c>
-      <c r="E35" t="inlineStr">
+      <c r="D36" t="n">
+        <v>59</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2025
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E195"/>
+  <dimension ref="A1:E215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:56:34</t>
+          <t>Última actualización: 16:24:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 190</t>
+          <t>Total filas: 210</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4233,11 +4233,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>15:02:46</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>93</v>
+        <v>10</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>15:02:46</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>15:02:46</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:36</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>109</v>
+        <v>12</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>15:02:46</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>117</v>
+        <v>23</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,23 +5198,523 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>16:48</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>24</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>27</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
           <t>15:02:46</t>
         </is>
       </c>
-      <c r="B195" t="inlineStr">
+      <c r="B197" t="inlineStr">
         <is>
           <t>16:59</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr">
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>117</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>15:02:46</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D195" t="n">
+      <c r="D198" t="n">
         <v>117</v>
       </c>
-      <c r="E195" t="inlineStr">
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>36</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>36</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>40</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>17:12</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>48</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>57</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>60</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>60</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>69</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>71</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>71</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>17:41</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>77</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>84</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>84</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>17:51</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>87</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>95</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>96</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>18:12</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>108</v>
+      </c>
+      <c r="E215" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5231,7 +5731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5244,14 +5744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:56:34</t>
+          <t>Última actualización: 16:24:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -6060,7 +6560,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>14:49:31</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6074,7 +6574,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6102,6 +6602,81 @@
         <v>117</v>
       </c>
       <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>36</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>84</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>84</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6118,7 +6693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6131,14 +6706,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:56:34</t>
+          <t>Última actualización: 16:24:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -6897,7 +7472,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>15:56:34</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6911,7 +7486,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6939,6 +7514,31 @@
         <v>59</v>
       </c>
       <c r="E36" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>32</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2026
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E215"/>
+  <dimension ref="A1:E226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:24:04</t>
+          <t>Última actualización: 16:49:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 210</t>
+          <t>Total filas: 221</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>85</v>
+        <v>28</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5258,7 +5258,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>15:02:46</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>117</v>
+        <v>10</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,7 +5298,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5308,11 +5308,11 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5348,12 +5348,12 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5378,16 +5378,16 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>17:12</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,12 +5448,12 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:23</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -5462,7 +5462,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5478,16 +5478,16 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5503,16 +5503,16 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5528,16 +5528,16 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>87</v>
+        <v>47</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>95</v>
+        <v>52</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>96</v>
+        <v>58</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,23 +5698,298 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
+          <t>16:49:32</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>59</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
           <t>16:24:04</t>
         </is>
       </c>
-      <c r="B215" t="inlineStr">
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>84</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>16:49:32</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>17:51</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>62</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>16:49:32</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>70</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>16:49:32</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>71</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>16:49:32</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>18:11</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>82</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>16:49:32</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
         <is>
           <t>18:12</t>
         </is>
       </c>
-      <c r="C215" t="inlineStr">
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>83</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>16:24:04</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>18:12</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D215" t="n">
+      <c r="D222" t="n">
         <v>108</v>
       </c>
-      <c r="E215" t="inlineStr">
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>16:49:32</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>94</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>16:49:32</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>95</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>16:49:32</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>106</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>16:49:32</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>18:38</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>109</v>
+      </c>
+      <c r="E226" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5731,7 +6006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5744,14 +6019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:24:04</t>
+          <t>Última actualización: 16:49:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -6610,7 +6885,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6624,7 +6899,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6635,21 +6910,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -6677,6 +6952,31 @@
         <v>84</v>
       </c>
       <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>16:49:32</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>59</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6693,7 +6993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6706,14 +7006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:24:04</t>
+          <t>Última actualización: 16:49:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -7497,12 +7797,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15:56:34</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:49</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -7511,7 +7811,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -7522,23 +7822,73 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>15:56:34</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>59</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>16:24:04</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>16:56</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="D38" t="n">
         <v>32</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>16:49:32</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>18:26</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>97</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2027
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:49:32</t>
+          <t>Última actualización: 17:02:25</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4533,7 +4533,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>15:02:46</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>117</v>
+        <v>10</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>10</v>
+        <v>117</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,7 +5298,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5308,11 +5308,11 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5848,7 +5848,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -5858,11 +5858,11 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>83</v>
+        <v>108</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5883,11 +5883,11 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>108</v>
+        <v>83</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -6019,7 +6019,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:49:32</t>
+          <t>Última actualización: 17:02:25</t>
         </is>
       </c>
     </row>
@@ -7006,7 +7006,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:49:32</t>
+          <t>Última actualización: 17:02:25</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:02:25</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7886,7 +7886,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2028
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E226"/>
+  <dimension ref="A1:E244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:02:25</t>
+          <t>Última actualización: 17:45:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 221</t>
+          <t>Total filas: 239</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>85</v>
+        <v>28</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4233,11 +4233,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>10</v>
+        <v>117</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>15:02:46</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>117</v>
+        <v>10</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:46</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>59</v>
+        <v>1</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:46</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5753,16 +5753,16 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:48</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5803,16 +5803,16 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:48</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>17:51</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>82</v>
+        <v>6</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>108</v>
+        <v>14</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5878,16 +5878,16 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>94</v>
+        <v>16</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:03</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>95</v>
+        <v>18</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5953,16 +5953,16 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,23 +5973,473 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>18:12</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>27</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>18:12</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>27</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>38</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>39</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>50</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>50</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
           <t>16:49:32</t>
         </is>
       </c>
-      <c r="B226" t="inlineStr">
+      <c r="B232" t="inlineStr">
         <is>
           <t>18:38</t>
         </is>
       </c>
-      <c r="C226" t="inlineStr">
+      <c r="C232" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D226" t="n">
+      <c r="D232" t="n">
         <v>109</v>
       </c>
-      <c r="E226" t="inlineStr">
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>18:39</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>54</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>18:41</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>56</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>18:51</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>66</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>68</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>75</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>19:09</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>84</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>87</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>92</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>98</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>99</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>111</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>115</v>
+      </c>
+      <c r="E244" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6006,7 +6456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6019,14 +6469,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:02:25</t>
+          <t>Última actualización: 17:45:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -6910,21 +7360,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -6935,12 +7385,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -6949,7 +7399,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -6977,6 +7427,81 @@
         <v>59</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>3</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>99</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>17:45:10</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>111</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7006,7 +7531,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:02:25</t>
+          <t>Última actualización: 17:45:10</t>
         </is>
       </c>
     </row>
@@ -7872,7 +8397,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>17:02:25</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7886,7 +8411,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>84</v>
+        <v>41</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2029
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E244"/>
+  <dimension ref="A1:E253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:45:10</t>
+          <t>Última actualización: 18:03:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 239</t>
+          <t>Total filas: 248</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4233,11 +4233,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5733,7 +5733,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D216" t="n">
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>82</v>
+        <v>1</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,12 +5973,12 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6012,7 +6012,7 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6028,16 +6028,16 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:33</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>18:38</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>109</v>
+        <v>50</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>18:41</t>
+          <t>18:38</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6203,16 +6203,16 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>18:39</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>75</v>
+        <v>48</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>19:09</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:01</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>92</v>
+        <v>58</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>98</v>
+        <v>65</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6378,16 +6378,16 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:09</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>111</v>
+        <v>69</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,23 +6423,248 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>19:14</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>71</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
           <t>17:45:10</t>
         </is>
       </c>
-      <c r="B244" t="inlineStr">
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>92</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>80</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>81</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>93</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
         <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="C244" t="inlineStr">
+      <c r="C249" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D244" t="n">
-        <v>115</v>
-      </c>
-      <c r="E244" t="inlineStr">
+      <c r="D249" t="n">
+        <v>97</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>104</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>19:53</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>110</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>19:54</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>111</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>117</v>
+      </c>
+      <c r="E253" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6469,7 +6694,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:45:10</t>
+          <t>Última actualización: 18:03:33</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7685,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7474,7 +7699,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -7485,7 +7710,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7499,7 +7724,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -7518,7 +7743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7531,14 +7756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:45:10</t>
+          <t>Última actualización: 18:03:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -8416,6 +8641,31 @@
       <c r="E39" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>75</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2030
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E253"/>
+  <dimension ref="A1:E269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:03:33</t>
+          <t>Última actualización: 18:39:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 248</t>
+          <t>Total filas: 264</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4233,11 +4233,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>15:02:46</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>117</v>
+        <v>10</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>10</v>
+        <v>117</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D207" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5733,7 +5733,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D216" t="n">
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>18:41</t>
+          <t>18:40</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6253,16 +6253,16 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:48</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>19:01</t>
+          <t>18:52</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6353,16 +6353,16 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>19:09</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>84</v>
+        <v>21</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:01</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>69</v>
+        <v>22</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,21 +6423,21 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>19:03</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>71</v>
+        <v>24</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>92</v>
+        <v>29</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:09</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>81</v>
+        <v>33</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6528,16 +6528,16 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>93</v>
+        <v>71</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,21 +6598,21 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>110</v>
+        <v>42</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>111</v>
+        <v>43</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6653,18 +6653,418 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>80</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>81</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>19:29</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>50</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>56</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>56</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>93</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>19:39</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>60</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>97</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>68</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>19:52</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>73</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>18:03:33</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>19:53</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>110</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>19:54</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>75</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
           <t>20:00</t>
         </is>
       </c>
-      <c r="C253" t="inlineStr">
+      <c r="C265" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D253" t="n">
-        <v>117</v>
-      </c>
-      <c r="E253" t="inlineStr">
+      <c r="D265" t="n">
+        <v>81</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>20:04</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>85</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>95</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>107</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>20:34</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>115</v>
+      </c>
+      <c r="E269" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6681,7 +7081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6694,14 +7094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:03:33</t>
+          <t>Última actualización: 18:39:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -7710,23 +8110,98 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>19:29</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>50</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>56</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>18:03:33</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>19:36</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D45" t="n">
+      <c r="D47" t="n">
         <v>93</v>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>95</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7743,7 +8218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7756,14 +8231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:03:33</t>
+          <t>Última actualización: 18:39:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -8647,23 +9122,48 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>38</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>18:03:33</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>19:18</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="D41" t="n">
         <v>75</v>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2031
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E269"/>
+  <dimension ref="A1:E280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:39:55</t>
+          <t>Última actualización: 18:57:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 264</t>
+          <t>Total filas: 275</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4233,11 +4233,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D207" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:57</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>19:01</t>
+          <t>18:58</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,21 +6423,21 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>19:03</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:01</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>19:09</t>
+          <t>19:03</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>84</v>
+        <v>24</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6503,16 +6503,16 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,21 +6523,21 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>19:09</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,12 +6573,12 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -6587,7 +6587,7 @@
         </is>
       </c>
       <c r="D250" t="n">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6603,16 +6603,16 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>80</v>
+        <v>24</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,21 +6673,21 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>19:29</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,21 +6723,21 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6753,16 +6753,16 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>19:29</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:33</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>93</v>
+        <v>36</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6803,16 +6803,16 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>19:39</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,21 +6823,21 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:39:55</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>97</v>
+        <v>56</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,21 +6848,21 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:36</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6878,16 +6878,16 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>19:52</t>
+          <t>19:39</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,21 +6898,21 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>110</v>
+        <v>43</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>81</v>
+        <v>50</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6978,16 +6978,16 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>20:04</t>
+          <t>19:52</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>95</v>
+        <v>56</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7028,16 +7028,16 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>19:54</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>107</v>
+        <v>75</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,23 +7048,298 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>58</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>63</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
           <t>18:39:55</t>
         </is>
       </c>
-      <c r="B269" t="inlineStr">
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>20:04</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>85</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>68</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>95</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>78</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>107</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>90</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>18:39:55</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
         <is>
           <t>20:34</t>
         </is>
       </c>
-      <c r="C269" t="inlineStr">
+      <c r="C277" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D269" t="n">
+      <c r="D277" t="n">
         <v>115</v>
       </c>
-      <c r="E269" t="inlineStr">
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>98</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>107</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>119</v>
+      </c>
+      <c r="E280" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7081,7 +7356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7094,14 +7369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:39:55</t>
+          <t>Última actualización: 18:57:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -8160,7 +8435,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8174,7 +8449,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>93</v>
+        <v>39</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -8185,23 +8460,123 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>50</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>18:39:55</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>20:14</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D48" t="n">
+      <c r="D49" t="n">
         <v>95</v>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>78</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>107</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>119</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8231,7 +8606,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:39:55</t>
+          <t>Última actualización: 18:57:14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2032
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E280"/>
+  <dimension ref="A1:E289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:57:14</t>
+          <t>Última actualización: 19:21:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 275</t>
+          <t>Total filas: 284</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>10</v>
+        <v>117</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>15:02:46</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>117</v>
+        <v>10</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,7 +5298,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5308,11 +5308,11 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D207" t="n">
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6673,7 +6673,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6687,7 +6687,7 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6773,7 +6773,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -6787,7 +6787,7 @@
         </is>
       </c>
       <c r="D258" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,7 +6798,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -6812,7 +6812,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6887,7 +6887,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>19:52</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,12 +6998,12 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:52</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -7012,7 +7012,7 @@
         </is>
       </c>
       <c r="D267" t="n">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,21 +7023,21 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,12 +7048,12 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:54</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -7062,7 +7062,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7078,16 +7078,16 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,21 +7098,21 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>20:04</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>85</v>
+        <v>38</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7128,16 +7128,16 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7153,16 +7153,16 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:04</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7178,16 +7178,16 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,21 +7198,21 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>107</v>
+        <v>45</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>90</v>
+        <v>49</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>20:34</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>115</v>
+        <v>49</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7303,16 +7303,16 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>107</v>
+        <v>78</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,23 +7323,248 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
+          <t>19:21:56</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>65</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
           <t>18:57:14</t>
         </is>
       </c>
-      <c r="B280" t="inlineStr">
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>90</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>19:21:56</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>20:34</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>73</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>98</v>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>19:21:56</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>20:43</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>82</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>107</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>19:21:56</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>20:49</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>88</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>19:21:56</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>94</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>19:21:56</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>94</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
         <is>
           <t>20:56</t>
         </is>
       </c>
-      <c r="C280" t="inlineStr">
+      <c r="C289" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D280" t="n">
+      <c r="D289" t="n">
         <v>119</v>
       </c>
-      <c r="E280" t="inlineStr">
+      <c r="E289" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7356,7 +7581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7369,14 +7594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:57:14</t>
+          <t>Última actualización: 19:21:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -8410,7 +8635,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8424,7 +8649,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8485,12 +8710,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>18:39:55</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -8499,7 +8724,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>95</v>
+        <v>49</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -8510,12 +8735,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -8524,7 +8749,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -8540,16 +8765,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>107</v>
+        <v>78</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -8560,23 +8785,98 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>19:21:56</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>20:43</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>82</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>18:57:14</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>107</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>19:21:56</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>94</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>18:57:14</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
         <is>
           <t>20:56</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D52" t="n">
+      <c r="D55" t="n">
         <v>119</v>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8606,7 +8906,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:57:14</t>
+          <t>Última actualización: 19:21:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2033
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E289"/>
+  <dimension ref="A1:E300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:21:56</t>
+          <t>Última actualización: 19:52:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 284</t>
+          <t>Total filas: 295</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>28</v>
+        <v>85</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>85</v>
+        <v>28</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4533,7 +4533,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>15:02:46</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>117</v>
+        <v>10</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>10</v>
+        <v>117</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,7 +5298,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5308,11 +5308,11 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5733,7 +5733,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D216" t="n">
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6998,7 +6998,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -7012,7 +7012,7 @@
         </is>
       </c>
       <c r="D267" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7048,7 +7048,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -7062,7 +7062,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7137,7 +7137,7 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>63</v>
+        <v>8</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7223,7 +7223,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -7233,11 +7233,11 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7258,7 +7258,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D277" t="n">
@@ -7278,7 +7278,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -7287,7 +7287,7 @@
         </is>
       </c>
       <c r="D278" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,21 +7298,21 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:11</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,21 +7323,21 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>65</v>
+        <v>22</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7353,16 +7353,16 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,21 +7373,21 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>20:34</t>
+          <t>20:18</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>98</v>
+        <v>34</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>20:43</t>
+          <t>20:27</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>107</v>
+        <v>39</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,21 +7473,21 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>20:49</t>
+          <t>20:34</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>88</v>
+        <v>42</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7528,16 +7528,16 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:43</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,23 +7548,298 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>52</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>19:21:56</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>20:49</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>88</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>59</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>20:52</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>60</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>63</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>19:21:56</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>94</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
           <t>18:57:14</t>
         </is>
       </c>
-      <c r="B289" t="inlineStr">
+      <c r="B295" t="inlineStr">
         <is>
           <t>20:56</t>
         </is>
       </c>
-      <c r="C289" t="inlineStr">
+      <c r="C295" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D289" t="n">
+      <c r="D295" t="n">
         <v>119</v>
       </c>
-      <c r="E289" t="inlineStr">
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>20:58</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>66</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>21:23</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>91</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>92</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>117</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>117</v>
+      </c>
+      <c r="E300" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7581,7 +7856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7594,14 +7869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:21:56</t>
+          <t>Última actualización: 19:52:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 51</t>
         </is>
       </c>
     </row>
@@ -8535,7 +8810,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8545,11 +8820,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8560,7 +8835,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -8570,11 +8845,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -8735,7 +9010,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -8749,7 +9024,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -8785,21 +9060,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>20:43</t>
+          <t>20:18</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -8810,12 +9085,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:43</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -8824,7 +9099,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>107</v>
+        <v>82</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -8835,21 +9110,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -8860,23 +9135,48 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>63</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>18:57:14</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>20:56</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D55" t="n">
+      <c r="D56" t="n">
         <v>119</v>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8893,7 +9193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8906,14 +9206,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:21:56</t>
+          <t>Última actualización: 19:52:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -9841,6 +10141,31 @@
       <c r="E41" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>104</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2034
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E300"/>
+  <dimension ref="A1:E309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:50</t>
+          <t>Última actualización: 20:20:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 295</t>
+          <t>Total filas: 304</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>85</v>
+        <v>28</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4233,11 +4233,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>10</v>
+        <v>117</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>15:02:46</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>117</v>
+        <v>10</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,7 +5298,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5308,11 +5308,11 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D207" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -7258,7 +7258,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D277" t="n">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D278" t="n">
@@ -7423,7 +7423,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>20:20:01</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -7437,7 +7437,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>90</v>
+        <v>7</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,12 +7448,12 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>20:20:01</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>20:31</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -7462,7 +7462,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7478,16 +7478,16 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>20:34</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>20:20:01</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:33</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>98</v>
+        <v>13</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>20:43</t>
+          <t>20:34</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>82</v>
+        <v>42</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,21 +7548,21 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>52</v>
+        <v>98</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>20:20:01</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>20:49</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>88</v>
+        <v>16</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,21 +7598,21 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:43</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7628,16 +7628,16 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>20:52</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,21 +7648,21 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>20:20:01</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7678,16 +7678,16 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:49</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,21 +7698,21 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>20:20:01</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>119</v>
+        <v>31</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7728,16 +7728,16 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>20:58</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>21:23</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7778,16 +7778,16 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>92</v>
+        <v>63</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>20:20:01</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>117</v>
+        <v>36</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,23 +7823,248 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
+          <t>20:20:01</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>37</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
           <t>19:52:50</t>
         </is>
       </c>
-      <c r="B300" t="inlineStr">
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>20:58</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>66</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>21:23</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>91</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>20:20:01</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>64</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>92</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>20:20:01</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>66</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>20:20:01</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>71</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
         <is>
           <t>21:49</t>
         </is>
       </c>
-      <c r="C300" t="inlineStr">
+      <c r="C307" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D300" t="n">
+      <c r="D307" t="n">
         <v>117</v>
       </c>
-      <c r="E300" t="inlineStr">
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>117</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>20:20:01</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>21:50</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>90</v>
+      </c>
+      <c r="E309" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7856,7 +8081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7869,14 +8094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:50</t>
+          <t>Última actualización: 20:20:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 51</t>
+          <t>Total filas: 52</t>
         </is>
       </c>
     </row>
@@ -8810,7 +9035,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8820,11 +9045,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8835,7 +9060,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -8845,11 +9070,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -9135,21 +9360,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>20:20:01</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -9160,23 +9385,48 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>63</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>20:20:01</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>20:56</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D56" t="n">
-        <v>119</v>
-      </c>
-      <c r="E56" t="inlineStr">
+      <c r="D57" t="n">
+        <v>36</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9193,7 +9443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9206,14 +9456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:50</t>
+          <t>Última actualización: 20:20:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -10147,25 +10397,100 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>20:20:01</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>25</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>19:52:50</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>21:36</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D43" t="n">
         <v>104</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>20:20:01</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>77</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>20:20:01</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>112</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2035
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:20:01</t>
+          <t>Última actualización: 20:49:20</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>85</v>
+        <v>28</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4233,11 +4233,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>15:02:46</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>117</v>
+        <v>10</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>15:02:46</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>10</v>
+        <v>117</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -7748,7 +7748,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
@@ -7758,11 +7758,11 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>94</v>
+        <v>63</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,7 +7773,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
@@ -7783,11 +7783,11 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>63</v>
+        <v>94</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7898,7 +7898,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>20:20:01</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
@@ -7908,11 +7908,11 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7923,7 +7923,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>20:20:01</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
@@ -7933,11 +7933,11 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -8094,7 +8094,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:20:01</t>
+          <t>Última actualización: 20:49:20</t>
         </is>
       </c>
     </row>
@@ -9443,7 +9443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9456,14 +9456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:20:01</t>
+          <t>Última actualización: 20:49:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -10447,7 +10447,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>20:20:01</t>
+          <t>20:49:20</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -10461,7 +10461,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>77</v>
+        <v>48</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -10472,7 +10472,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>20:20:01</t>
+          <t>20:49:20</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -10486,9 +10486,34 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>112</v>
+        <v>83</v>
       </c>
       <c r="E45" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>20:49:20</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>22:32</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>103</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2036
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-28.xlsx
+++ b/data/horarios-141-2026-03-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E309"/>
+  <dimension ref="A1:E319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:49:20</t>
+          <t>Última actualización: 21:03:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 304</t>
+          <t>Total filas: 314</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07:57:31</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,11 +983,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>07:57:31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:48:26</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1483,11 +1483,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>08:48:26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1508,11 +1508,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>12:51:43</t>
+          <t>12:24:27</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>11:27:21</t>
+          <t>12:51:43</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>12:24:27</t>
+          <t>11:27:21</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>28</v>
+        <v>85</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>13:20:14</t>
+          <t>13:53:51</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:53:51</t>
+          <t>13:20:14</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -5298,7 +5298,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5308,11 +5308,11 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D207" t="n">
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>16:24:04</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>16:24:04</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:49:32</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5783,11 +5783,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>16:49:32</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5808,11 +5808,11 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>18:03:33</t>
+          <t>17:45:10</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>17:45:10</t>
+          <t>18:03:33</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6158,11 +6158,11 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6948,7 +6948,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>18:57:14</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -6958,11 +6958,11 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,7 +6973,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>18:57:14</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -6983,11 +6983,11 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -7223,7 +7223,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>19:21:56</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -7233,11 +7233,11 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7258,7 +7258,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D277" t="n">
@@ -7273,7 +7273,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>19:21:56</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -7283,11 +7283,11 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7873,21 +7873,21 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>21:03:38</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>21:23</t>
+          <t>21:22</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>91</v>
+        <v>19</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -7898,21 +7898,21 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>21:03:38</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>21:23</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>92</v>
+        <v>20</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7948,12 +7948,12 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>20:20:01</t>
+          <t>19:52:50</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:24</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -7962,7 +7962,7 @@
         </is>
       </c>
       <c r="D305" t="n">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,21 +7973,21 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>20:20:01</t>
+          <t>21:03:38</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>21:31</t>
+          <t>21:25</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>71</v>
+        <v>22</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -7998,21 +7998,21 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>20:20:01</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:26</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>117</v>
+        <v>66</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>21:03:38</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>117</v>
+        <v>27</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8053,18 +8053,268 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>71</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>21:03:38</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>46</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>19:52:50</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>117</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>20:20:01</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
           <t>21:50</t>
         </is>
       </c>
-      <c r="C309" t="inlineStr">
+      <c r="C312" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D309" t="n">
+      <c r="D312" t="n">
         <v>90</v>
       </c>
-      <c r="E309" t="inlineStr">
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>21:03:38</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>21:50</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>47</v>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>21:03:38</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>69</v>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>21:03:38</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>22:19</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>76</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>21:03:38</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>22:23</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D316" t="n">
+        <v>80</v>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>21:03:38</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>83</v>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>21:03:38</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>22:49</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>106</v>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>21:03:38</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>22:59</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>116</v>
+      </c>
+      <c r="E319" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8081,7 +8331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8094,14 +8344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:49:20</t>
+          <t>Última actualización: 21:03:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 52</t>
+          <t>Total filas: 53</t>
         </is>
       </c>
     </row>
@@ -9427,6 +9677,31 @@
         <v>36</v>
       </c>
       <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>21:03:38</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>83</v>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9456,7 +9731,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:49:20</t>
+          <t>Última actualización: 21:03:38</t>
         </is>
       </c>
     </row>
@@ -10422,7 +10697,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>19:52:50</t>
+          <t>21:03:38</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -10436,7 +10711,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>104</v>
+        <v>33</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -10472,7 +10747,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>20:49:20</t>
+          <t>21:03:38</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -10486,7 +10761,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -10497,7 +10772,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>20:49:20</t>
+          <t>21:03:38</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -10511,7 +10786,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>

</xml_diff>